<commit_message>
actualiza calendario (63->65) y corrige matcher de GPX
- Excel editado + GPX/TCX nuevos: Los Lenos ... cuesta zapata (base y Capu),
  y Lo Prado - Ibacache -Quintay ( Ristretto + Macchiato)
- getFileIndex: coincidencia exacta por nombre base (stem) + fallback difuso al mas corto;
  arregla que la ruta 24/10 agarrara "... Capu.gpx" en vez del archivo base
- Waze/Maps se recalculan del inicio del GPX (24/10 y Quintay correctos)
- validacion limpia: GPX no encontrados 0, 65 rutas, 97 usuarios

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013BB8FF-DD14-E145-98F9-8B8ABA873EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF9F264-85DD-8642-A182-E50A0FCD860E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="382">
   <si>
     <t>Fecha</t>
   </si>
@@ -1126,9 +1126,6 @@
     <t>Aurora - Cuesta Barriga - Cuesta Mallarauco - Chorombo</t>
   </si>
   <si>
-    <t>Kross - Pangue - Casa Blanca - Cuesta Zapata - Kross</t>
-  </si>
-  <si>
     <t>68 Ribs - Pangue - Casablanca - La Playa - Cuesta Zapata - 68 Ribs</t>
   </si>
   <si>
@@ -1169,6 +1166,24 @@
   </si>
   <si>
     <t>10.652.669-9</t>
+  </si>
+  <si>
+    <t>Los Leños</t>
+  </si>
+  <si>
+    <t>Los Leños - Pangue - Casa Blanca - Cuesta Zapata - Los Leños</t>
+  </si>
+  <si>
+    <t>Los Leños - Pangue - casa blanca - Geronimo - cuesta zapata</t>
+  </si>
+  <si>
+    <t>Quintay</t>
+  </si>
+  <si>
+    <t>Lo Prado - Ibacache -Quintay</t>
+  </si>
+  <si>
+    <t>Lo Prado - Ibacache -Quintay  ( Ristretto + Macchiato).gpx</t>
   </si>
 </sst>
 </file>
@@ -1660,7 +1675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" style="6" customWidth="1"/>
@@ -1690,13 +1705,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>372</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>373</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
@@ -2428,7 +2443,7 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>36</v>
@@ -2792,7 +2807,7 @@
         <v>358</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>36</v>
@@ -2874,7 +2889,7 @@
         <v>360</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E43" s="7" t="s">
         <v>36</v>
@@ -2928,7 +2943,7 @@
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>36</v>
@@ -3034,7 +3049,7 @@
         <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D49" s="28" t="s">
         <v>29</v>
@@ -3047,10 +3062,10 @@
         <v>Strava</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="H49" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -3061,7 +3076,7 @@
         <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D50" t="s">
         <v>70</v>
@@ -3116,23 +3131,23 @@
         <v>5</v>
       </c>
       <c r="C52" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="D52" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="E52" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F52" s="7" t="str">
-        <f t="shared" ref="F52" si="47">E52</f>
+        <f t="shared" ref="F52:F53" si="47">E52</f>
         <v>Strava</v>
       </c>
       <c r="G52" s="7" t="s">
         <v>36</v>
       </c>
       <c r="H52" t="s">
-        <v>362</v>
+        <v>378</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -3143,23 +3158,24 @@
         <v>5</v>
       </c>
       <c r="C53" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D53" t="s">
-        <v>366</v>
+        <v>31</v>
       </c>
       <c r="E53" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F53" s="7" t="str">
-        <f t="shared" ref="F53" si="48">E53</f>
-        <v>Strava</v>
-      </c>
-      <c r="G53" s="7" t="s">
-        <v>36</v>
+        <f t="shared" si="47"/>
+        <v>Strava</v>
+      </c>
+      <c r="G53" s="7" t="str">
+        <f t="shared" ref="G53" si="48">F53</f>
+        <v>Strava</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -3170,10 +3186,10 @@
         <v>6</v>
       </c>
       <c r="C54" t="s">
-        <v>18</v>
+        <v>380</v>
       </c>
       <c r="D54" t="s">
-        <v>33</v>
+        <v>379</v>
       </c>
       <c r="E54" s="7" t="s">
         <v>36</v>
@@ -3186,7 +3202,7 @@
         <v>36</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>62</v>
+        <v>381</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -3252,10 +3268,10 @@
         <v>5</v>
       </c>
       <c r="C57" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D57" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>36</v>
@@ -3268,7 +3284,7 @@
         <v>36</v>
       </c>
       <c r="H57" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -3279,7 +3295,7 @@
         <v>6</v>
       </c>
       <c r="C58" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D58" t="s">
         <v>70</v>
@@ -3307,7 +3323,7 @@
         <v>6</v>
       </c>
       <c r="C59" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D59" t="s">
         <v>70</v>
@@ -3335,7 +3351,7 @@
         <v>6</v>
       </c>
       <c r="C60" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D60" t="s">
         <v>70</v>
@@ -3360,10 +3376,10 @@
         <v>46361</v>
       </c>
       <c r="B61" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C61" s="29" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D61" t="s">
         <v>26</v>
@@ -3379,7 +3395,7 @@
         <v>36</v>
       </c>
       <c r="H61" s="29" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -3390,7 +3406,7 @@
         <v>5</v>
       </c>
       <c r="C62" s="29" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D62" t="s">
         <v>29</v>
@@ -3406,7 +3422,7 @@
         <v>36</v>
       </c>
       <c r="H62" s="29" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -3453,7 +3469,7 @@
         <v>36</v>
       </c>
       <c r="F64" s="7" t="str">
-        <f t="shared" ref="F64" si="59">E64</f>
+        <f t="shared" ref="F64:F66" si="59">E64</f>
         <v>Strava</v>
       </c>
       <c r="G64" s="7" t="s">
@@ -3461,6 +3477,61 @@
       </c>
       <c r="H64" s="2" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" s="6">
+        <v>46392</v>
+      </c>
+      <c r="B65" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" t="s">
+        <v>16</v>
+      </c>
+      <c r="D65" t="s">
+        <v>31</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F65" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Strava</v>
+      </c>
+      <c r="G65" s="7" t="str">
+        <f t="shared" ref="G65" si="60">F65</f>
+        <v>Strava</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" s="6">
+        <v>46401</v>
+      </c>
+      <c r="B66" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" t="s">
+        <v>22</v>
+      </c>
+      <c r="D66" t="s">
+        <v>365</v>
+      </c>
+      <c r="E66" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F66" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Strava</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H66" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -3493,48 +3564,52 @@
     <hyperlink ref="E20" r:id="rId26" xr:uid="{8866888E-71DF-3944-9620-4E948829D43F}"/>
     <hyperlink ref="E25" r:id="rId27" xr:uid="{F67F5632-1B2B-C049-8C5C-D8F9CF9A87E3}"/>
     <hyperlink ref="E24" r:id="rId28" xr:uid="{F51A13EB-7897-0D42-A463-97945F82F47E}"/>
-    <hyperlink ref="E53" r:id="rId29" xr:uid="{8F50E81C-F18A-CE4F-A98D-3D4F1A293290}"/>
-    <hyperlink ref="E54" r:id="rId30" xr:uid="{B1BBA9B4-EBD6-9343-BDD3-B3D8AA59AD32}"/>
-    <hyperlink ref="E55" r:id="rId31" xr:uid="{BAEB0B98-6FB1-434C-B4D4-0C351FA1E8AA}"/>
-    <hyperlink ref="E56" r:id="rId32" xr:uid="{A1058D29-89CB-8B47-A38D-E24CFFAD7387}"/>
-    <hyperlink ref="E64" r:id="rId33" xr:uid="{0A9781F8-06DF-AD4B-8C0E-450CBD0E1ED5}"/>
-    <hyperlink ref="E39" r:id="rId34" xr:uid="{5D621643-1857-6949-A5EE-8D21ACA6D173}"/>
-    <hyperlink ref="E48" r:id="rId35" xr:uid="{28C15F8B-DF41-8E47-BE95-3FF9ADA04A9D}"/>
-    <hyperlink ref="E46" r:id="rId36" xr:uid="{050206DA-2A1C-9247-B538-A6C21B74792C}"/>
-    <hyperlink ref="E51" r:id="rId37" xr:uid="{DDF27CF3-067C-2C40-831B-B30E6A059FA4}"/>
-    <hyperlink ref="E42" r:id="rId38" xr:uid="{5FE6AEA5-9829-0A4C-901D-15C508BE82B4}"/>
-    <hyperlink ref="E38" r:id="rId39" xr:uid="{7D056CB1-8218-B047-8B01-6450203D5916}"/>
-    <hyperlink ref="E47" r:id="rId40" xr:uid="{72C58610-12F4-3347-94C5-89094846F7BC}"/>
-    <hyperlink ref="E63" r:id="rId41" xr:uid="{3081F97D-82DE-804B-AF13-E78A89A26914}"/>
-    <hyperlink ref="E49" r:id="rId42" xr:uid="{9AEFB797-EACB-874E-98CC-22F5AB6C6FDF}"/>
-    <hyperlink ref="E44" r:id="rId43" xr:uid="{6DE013C7-DC12-5045-8866-5F063A0E4BBC}"/>
-    <hyperlink ref="E36" r:id="rId44" xr:uid="{8ABC89D8-C10E-0C45-833D-F730BBEC276D}"/>
-    <hyperlink ref="E37" r:id="rId45" xr:uid="{610CEF98-CEDF-3B46-95F5-F415021045BC}"/>
-    <hyperlink ref="E40" r:id="rId46" xr:uid="{2B098DA7-1C63-7346-BDC5-428B06DB46E4}"/>
-    <hyperlink ref="E43" r:id="rId47" xr:uid="{E7F94F05-CCA9-B043-B789-CE3339CC6812}"/>
-    <hyperlink ref="E52" r:id="rId48" xr:uid="{C00B5D1B-6D1B-5F46-9E19-728B32AD9191}"/>
-    <hyperlink ref="E57" r:id="rId49" xr:uid="{C923ADC7-05BB-7744-8BF3-B3DF402E49A0}"/>
-    <hyperlink ref="E61" r:id="rId50" xr:uid="{583CF50F-498E-0841-9BC9-5A9E3F837061}"/>
-    <hyperlink ref="E62" r:id="rId51" xr:uid="{030FBD56-AB0C-764C-BC0B-06F85764D9FD}"/>
-    <hyperlink ref="E45" r:id="rId52" xr:uid="{5BD7D123-7286-5A47-A0D9-8170243675C4}"/>
-    <hyperlink ref="G40" r:id="rId53" xr:uid="{8B72540D-E184-594B-B7BB-931E8CE8066C}"/>
-    <hyperlink ref="G42" r:id="rId54" xr:uid="{FF907A16-C49B-6940-9A49-5174184D91E8}"/>
-    <hyperlink ref="G43" r:id="rId55" xr:uid="{80F54F31-0D14-BA40-9830-6A3A4B290D55}"/>
-    <hyperlink ref="G44" r:id="rId56" xr:uid="{8D267D2E-3A23-4B48-B88F-051285D7BA36}"/>
-    <hyperlink ref="G46" r:id="rId57" xr:uid="{361489AA-38BC-2442-A548-A3F7EDFC8002}"/>
-    <hyperlink ref="G47" r:id="rId58" xr:uid="{5F56807E-FBB9-7144-8BED-5D4FB192A8EE}"/>
-    <hyperlink ref="G48" r:id="rId59" xr:uid="{5363C3C8-9072-9A44-983D-1FD0E3428E68}"/>
-    <hyperlink ref="G49" r:id="rId60" xr:uid="{549A2681-C267-8E45-844F-EF310CCCFDB2}"/>
-    <hyperlink ref="G51" r:id="rId61" xr:uid="{63252D4C-E3AC-1148-8CA9-B56CCD344D36}"/>
-    <hyperlink ref="G52" r:id="rId62" xr:uid="{98440C2B-FB64-3B47-868F-4D555F1A88B1}"/>
-    <hyperlink ref="G53" r:id="rId63" xr:uid="{EBCB25C5-25F2-8847-BE10-5DC3A3FB264F}"/>
-    <hyperlink ref="G54" r:id="rId64" xr:uid="{9C5D2F10-3E58-BB41-B927-BFF3018F1450}"/>
-    <hyperlink ref="G56" r:id="rId65" xr:uid="{A7AA9CE7-D397-ED45-A134-D461653F928E}"/>
-    <hyperlink ref="G57" r:id="rId66" xr:uid="{54BD7C89-AE76-544E-ACFF-B6F9DDAB007A}"/>
-    <hyperlink ref="G61" r:id="rId67" xr:uid="{1A12B0E4-5936-BD49-B04D-141DE949D1CB}"/>
-    <hyperlink ref="G62" r:id="rId68" xr:uid="{676807D1-D959-964B-B19D-ABBB412ECB83}"/>
-    <hyperlink ref="G63" r:id="rId69" xr:uid="{55193CD3-AD02-9F4A-A96B-72D44533BB4F}"/>
-    <hyperlink ref="G64" r:id="rId70" xr:uid="{D1B99FE7-3D04-C048-9F49-E9DE3DCBD207}"/>
+    <hyperlink ref="E54" r:id="rId29" xr:uid="{B1BBA9B4-EBD6-9343-BDD3-B3D8AA59AD32}"/>
+    <hyperlink ref="E55" r:id="rId30" xr:uid="{BAEB0B98-6FB1-434C-B4D4-0C351FA1E8AA}"/>
+    <hyperlink ref="E56" r:id="rId31" xr:uid="{A1058D29-89CB-8B47-A38D-E24CFFAD7387}"/>
+    <hyperlink ref="E64" r:id="rId32" xr:uid="{0A9781F8-06DF-AD4B-8C0E-450CBD0E1ED5}"/>
+    <hyperlink ref="E39" r:id="rId33" xr:uid="{5D621643-1857-6949-A5EE-8D21ACA6D173}"/>
+    <hyperlink ref="E48" r:id="rId34" xr:uid="{28C15F8B-DF41-8E47-BE95-3FF9ADA04A9D}"/>
+    <hyperlink ref="E46" r:id="rId35" xr:uid="{050206DA-2A1C-9247-B538-A6C21B74792C}"/>
+    <hyperlink ref="E51" r:id="rId36" xr:uid="{DDF27CF3-067C-2C40-831B-B30E6A059FA4}"/>
+    <hyperlink ref="E42" r:id="rId37" xr:uid="{5FE6AEA5-9829-0A4C-901D-15C508BE82B4}"/>
+    <hyperlink ref="E38" r:id="rId38" xr:uid="{7D056CB1-8218-B047-8B01-6450203D5916}"/>
+    <hyperlink ref="E47" r:id="rId39" xr:uid="{72C58610-12F4-3347-94C5-89094846F7BC}"/>
+    <hyperlink ref="E63" r:id="rId40" xr:uid="{3081F97D-82DE-804B-AF13-E78A89A26914}"/>
+    <hyperlink ref="E49" r:id="rId41" xr:uid="{9AEFB797-EACB-874E-98CC-22F5AB6C6FDF}"/>
+    <hyperlink ref="E44" r:id="rId42" xr:uid="{6DE013C7-DC12-5045-8866-5F063A0E4BBC}"/>
+    <hyperlink ref="E36" r:id="rId43" xr:uid="{8ABC89D8-C10E-0C45-833D-F730BBEC276D}"/>
+    <hyperlink ref="E37" r:id="rId44" xr:uid="{610CEF98-CEDF-3B46-95F5-F415021045BC}"/>
+    <hyperlink ref="E40" r:id="rId45" xr:uid="{2B098DA7-1C63-7346-BDC5-428B06DB46E4}"/>
+    <hyperlink ref="E43" r:id="rId46" xr:uid="{E7F94F05-CCA9-B043-B789-CE3339CC6812}"/>
+    <hyperlink ref="E52" r:id="rId47" xr:uid="{C00B5D1B-6D1B-5F46-9E19-728B32AD9191}"/>
+    <hyperlink ref="E57" r:id="rId48" xr:uid="{C923ADC7-05BB-7744-8BF3-B3DF402E49A0}"/>
+    <hyperlink ref="E61" r:id="rId49" xr:uid="{583CF50F-498E-0841-9BC9-5A9E3F837061}"/>
+    <hyperlink ref="E62" r:id="rId50" xr:uid="{030FBD56-AB0C-764C-BC0B-06F85764D9FD}"/>
+    <hyperlink ref="E45" r:id="rId51" xr:uid="{5BD7D123-7286-5A47-A0D9-8170243675C4}"/>
+    <hyperlink ref="G40" r:id="rId52" xr:uid="{8B72540D-E184-594B-B7BB-931E8CE8066C}"/>
+    <hyperlink ref="G42" r:id="rId53" xr:uid="{FF907A16-C49B-6940-9A49-5174184D91E8}"/>
+    <hyperlink ref="G43" r:id="rId54" xr:uid="{80F54F31-0D14-BA40-9830-6A3A4B290D55}"/>
+    <hyperlink ref="G44" r:id="rId55" xr:uid="{8D267D2E-3A23-4B48-B88F-051285D7BA36}"/>
+    <hyperlink ref="G46" r:id="rId56" xr:uid="{361489AA-38BC-2442-A548-A3F7EDFC8002}"/>
+    <hyperlink ref="G47" r:id="rId57" xr:uid="{5F56807E-FBB9-7144-8BED-5D4FB192A8EE}"/>
+    <hyperlink ref="G48" r:id="rId58" xr:uid="{5363C3C8-9072-9A44-983D-1FD0E3428E68}"/>
+    <hyperlink ref="G49" r:id="rId59" xr:uid="{549A2681-C267-8E45-844F-EF310CCCFDB2}"/>
+    <hyperlink ref="G51" r:id="rId60" xr:uid="{63252D4C-E3AC-1148-8CA9-B56CCD344D36}"/>
+    <hyperlink ref="G52" r:id="rId61" xr:uid="{98440C2B-FB64-3B47-868F-4D555F1A88B1}"/>
+    <hyperlink ref="G54" r:id="rId62" xr:uid="{9C5D2F10-3E58-BB41-B927-BFF3018F1450}"/>
+    <hyperlink ref="G56" r:id="rId63" xr:uid="{A7AA9CE7-D397-ED45-A134-D461653F928E}"/>
+    <hyperlink ref="G57" r:id="rId64" xr:uid="{54BD7C89-AE76-544E-ACFF-B6F9DDAB007A}"/>
+    <hyperlink ref="G61" r:id="rId65" xr:uid="{1A12B0E4-5936-BD49-B04D-141DE949D1CB}"/>
+    <hyperlink ref="G62" r:id="rId66" xr:uid="{676807D1-D959-964B-B19D-ABBB412ECB83}"/>
+    <hyperlink ref="G63" r:id="rId67" xr:uid="{55193CD3-AD02-9F4A-A96B-72D44533BB4F}"/>
+    <hyperlink ref="G64" r:id="rId68" xr:uid="{D1B99FE7-3D04-C048-9F49-E9DE3DCBD207}"/>
+    <hyperlink ref="F52" r:id="rId69" display="https://www.strava.com/routes/3547364261272700544" xr:uid="{17DDA6E6-A166-C34C-BA54-08DBE09B057A}"/>
+    <hyperlink ref="F54" r:id="rId70" display="https://www.strava.com/routes/2921779823437514684" xr:uid="{A7312173-DDB6-D447-B1F7-15679E1CD753}"/>
+    <hyperlink ref="E65" r:id="rId71" xr:uid="{90DE291A-38D6-E242-8D90-7C935A61EE70}"/>
+    <hyperlink ref="E66" r:id="rId72" xr:uid="{D4478EC3-3290-4F43-90C2-5265AF0FBE32}"/>
+    <hyperlink ref="G66" r:id="rId73" xr:uid="{F10A536E-ADAA-524A-AFC3-4934163DDF1A}"/>
+    <hyperlink ref="E53" r:id="rId74" xr:uid="{FE6EEA27-F392-754C-91B9-6E47345C97F4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4512,7 +4587,7 @@
         <v>76</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D57" s="18" t="s">
         <v>219</v>

</xml_diff>

<commit_message>
agrega 4 socios a la hoja Usuarios (97 -> 101)
- Max Spiess, Rolando Libra, Daniela Salgado, Mario Gutierrez (todos PIN unico)
- se omite Alejandro Ihnen: ya existia (evita PIN duplicado 3422 que romperia su login)
- edicion quirurgica del XML preservando sharedStrings (openpyxl rompe el parser del server)
- verificado: 101 usuarios, 0 PIN duplicados, rutas intactas (65, GPX 0)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="394">
   <si>
     <t>Fecha</t>
   </si>
@@ -1184,6 +1184,42 @@
   </si>
   <si>
     <t>Lo Prado - Ibacache -Quintay  ( Ristretto + Macchiato).gpx</t>
+  </si>
+  <si>
+    <t>10.680.661-6</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Spiess</t>
+  </si>
+  <si>
+    <t>10.203.205-5</t>
+  </si>
+  <si>
+    <t>Rolando</t>
+  </si>
+  <si>
+    <t>Libra</t>
+  </si>
+  <si>
+    <t>15.899.064-4</t>
+  </si>
+  <si>
+    <t>Daniela</t>
+  </si>
+  <si>
+    <t>Salgado</t>
+  </si>
+  <si>
+    <t>13.642.444-0</t>
+  </si>
+  <si>
+    <t>Mario</t>
+  </si>
+  <si>
+    <t>Gutiérrez</t>
   </si>
 </sst>
 </file>
@@ -3617,7 +3653,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CA8C7-05A5-DA44-B969-9E41B832BB96}">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
@@ -5296,6 +5332,74 @@
         <v>318</v>
       </c>
     </row>
+    <row r="99" spans="1:5">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C99" s="22" t="s">
+        <v>382</v>
+      </c>
+      <c r="D99" s="23" t="s">
+        <v>383</v>
+      </c>
+      <c r="E99" s="23" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C100" s="22" t="s">
+        <v>385</v>
+      </c>
+      <c r="D100" s="23" t="s">
+        <v>386</v>
+      </c>
+      <c r="E100" s="23" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C101" s="22" t="s">
+        <v>388</v>
+      </c>
+      <c r="D101" s="23" t="s">
+        <v>389</v>
+      </c>
+      <c r="E101" s="23" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C102" s="22" t="s">
+        <v>391</v>
+      </c>
+      <c r="D102" s="23" t="s">
+        <v>392</v>
+      </c>
+      <c r="E102" s="23" t="s">
+        <v>393</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E98" xr:uid="{2B1CA8C7-05A5-DA44-B969-9E41B832BB96}"/>
   <hyperlinks>

</xml_diff>